<commit_message>
W9-04: Updated FY2025 upload, review, and reupload/version-history flow.
</commit_message>
<xml_diff>
--- a/test_samples/pr_batch_a_exact_copy_different_name.xlsx
+++ b/test_samples/pr_batch_a_exact_copy_different_name.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Raw Filtered Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,356 +425,598 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:AJ4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="35" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PR</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PO</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>PR Status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>PO Status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>VR</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Term Contract Number</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Purch Grp</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Req Type</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>PR Sub Date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Requestor</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Staff ID</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Division</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Procurement Basis</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>ITQ Ref</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>VendorEmail</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Curr</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Grand Total in SGD</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Item Details</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>UOM</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Unit Rate</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Delivery Date</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>MCA</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Allocatn</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>WBS</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>GL</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Fund Type</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Asset ID</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Part/Full Award</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>T&amp;C</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Reason for Waiver</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Instruction to Vendor</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>PR Category</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Lab</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Amount + GST</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PR-2026-2001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
+          <t>PR2500002001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sarah Chen</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>W3 food processing practical consumables</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1280.00</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Sterile sample containers</t>
-        </is>
-      </c>
+          <t>Pending Approval</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>LAB</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>12.00</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Randy Kwok</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>S1234567A</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Quotation</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Purchase consumables for W3 Food Processing Lab</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Lab Supplies Pte Ltd</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>sales@labsupplies.example</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1250.00</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Food-grade sample containers</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>box</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>25.00</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr">
+        <is>
           <t>WBS-FCB-001</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Deliver to W3 food processing lab</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Consumables</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>W3 Food Processing Lab</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>240.00</t>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>604001</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>MOE</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Deliver cartons to W3-01-021 storage area</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PR-2026-2001</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
+          <t>PR2500002002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sarah Chen</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>W3 food processing practical consumables</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1280.00</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Food-grade cleaning solution</t>
-        </is>
-      </c>
+          <t>Pending Approval</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>LAB</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>55.00</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>WBS-FCB-001</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Deliver to W3 food processing lab</t>
+          <t>Azzalia Abu</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Consumables</t>
+          <t>S7654321B</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>W3 Food Processing Lab</t>
+          <t>Infocomm</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>440.00</t>
+          <t>Quotation</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Embedded controller parts for ICT Embedded Lab</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Tech Parts Pte Ltd</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>orders@techparts.example</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>900.00</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Microcontroller evaluation boards</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>300.00</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>WBS-ICT-002</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>604002</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>MOE</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Deliver to E2-02-02 bench 4</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PR-2026-2002</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
+          <t>PR2500002003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Randy Kwok</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Software lab equipment refresh</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>3500.00</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Embedded systems training kits</t>
-        </is>
-      </c>
+          <t>Pending Approval</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>LAB</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>620.00</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>WBS-ICT-002</t>
+          <t>03/04/2026</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Deliver to software systems lab</t>
+          <t>Unknown Requestor</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>S1111111C</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Software Systems Lab</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>3100.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>PR-2026-2003</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Mei Tan</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>General workshop materials</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>650.00</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Miscellaneous workshop supplies</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>65.00</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>WBS-UNKNOWN-999</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Deliver to main office</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>650.00</t>
+          <t>Quotation</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>General lab supplies for upcoming practical</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>General Vendor Pte Ltd</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>hello@generalvendor.example</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>SGD</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>480.00</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Mixed consumables kit</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>604003</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>MOE</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Deliver to temporary holding room</t>
         </is>
       </c>
     </row>

</xml_diff>